<commit_message>
Atualizando arquivo de notas
</commit_message>
<xml_diff>
--- a/notas-chamada.xlsx
+++ b/notas-chamada.xlsx
@@ -2035,7 +2035,7 @@
     <numFmt numFmtId="172" formatCode="0.00"/>
     <numFmt numFmtId="173" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -2090,6 +2090,12 @@
       <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -2475,7 +2481,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2495,11 +2501,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2511,7 +2517,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2519,7 +2525,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2547,7 +2553,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2555,15 +2561,15 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="13" fillId="7" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="14" fillId="7" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2876,78 +2882,78 @@
       <c r="FZ4" s="1"/>
       <c r="GA4" s="1"/>
       <c r="GB4" s="1"/>
-      <c r="GC4" s="0"/>
-      <c r="GD4" s="0"/>
-      <c r="GE4" s="0"/>
-      <c r="GF4" s="0"/>
-      <c r="GG4" s="0"/>
-      <c r="GH4" s="0"/>
-      <c r="GI4" s="0"/>
-      <c r="GJ4" s="0"/>
-      <c r="GK4" s="0"/>
-      <c r="GL4" s="0"/>
-      <c r="GM4" s="0"/>
-      <c r="GN4" s="0"/>
-      <c r="GO4" s="0"/>
-      <c r="GP4" s="0"/>
-      <c r="GQ4" s="0"/>
-      <c r="GR4" s="0"/>
-      <c r="GS4" s="0"/>
-      <c r="GT4" s="0"/>
-      <c r="GU4" s="0"/>
-      <c r="GV4" s="0"/>
-      <c r="GW4" s="0"/>
-      <c r="GX4" s="0"/>
-      <c r="GY4" s="0"/>
-      <c r="GZ4" s="0"/>
-      <c r="HA4" s="0"/>
-      <c r="HB4" s="0"/>
-      <c r="HC4" s="0"/>
-      <c r="HD4" s="0"/>
-      <c r="HE4" s="0"/>
-      <c r="HF4" s="0"/>
-      <c r="HG4" s="0"/>
-      <c r="HH4" s="0"/>
-      <c r="HI4" s="0"/>
-      <c r="HJ4" s="0"/>
-      <c r="HK4" s="0"/>
-      <c r="HL4" s="0"/>
-      <c r="HM4" s="0"/>
-      <c r="HN4" s="0"/>
-      <c r="HO4" s="0"/>
-      <c r="HP4" s="0"/>
-      <c r="HQ4" s="0"/>
-      <c r="HR4" s="0"/>
-      <c r="HS4" s="0"/>
-      <c r="HT4" s="0"/>
-      <c r="HU4" s="0"/>
-      <c r="HV4" s="0"/>
-      <c r="HW4" s="0"/>
-      <c r="HX4" s="0"/>
-      <c r="HY4" s="0"/>
-      <c r="HZ4" s="0"/>
-      <c r="IA4" s="0"/>
-      <c r="IB4" s="0"/>
-      <c r="IC4" s="0"/>
-      <c r="ID4" s="0"/>
-      <c r="IE4" s="0"/>
-      <c r="IF4" s="0"/>
-      <c r="IG4" s="0"/>
-      <c r="IH4" s="0"/>
-      <c r="II4" s="0"/>
-      <c r="IJ4" s="0"/>
-      <c r="IK4" s="0"/>
-      <c r="IL4" s="0"/>
-      <c r="IM4" s="0"/>
-      <c r="IN4" s="0"/>
-      <c r="IO4" s="0"/>
-      <c r="IP4" s="0"/>
-      <c r="IQ4" s="0"/>
-      <c r="IR4" s="0"/>
-      <c r="IS4" s="0"/>
-      <c r="IT4" s="0"/>
-      <c r="IU4" s="0"/>
-      <c r="IV4" s="0"/>
+      <c r="GC4" s="1"/>
+      <c r="GD4" s="1"/>
+      <c r="GE4" s="1"/>
+      <c r="GF4" s="1"/>
+      <c r="GG4" s="1"/>
+      <c r="GH4" s="1"/>
+      <c r="GI4" s="1"/>
+      <c r="GJ4" s="1"/>
+      <c r="GK4" s="1"/>
+      <c r="GL4" s="1"/>
+      <c r="GM4" s="1"/>
+      <c r="GN4" s="1"/>
+      <c r="GO4" s="1"/>
+      <c r="GP4" s="1"/>
+      <c r="GQ4" s="1"/>
+      <c r="GR4" s="1"/>
+      <c r="GS4" s="1"/>
+      <c r="GT4" s="1"/>
+      <c r="GU4" s="1"/>
+      <c r="GV4" s="1"/>
+      <c r="GW4" s="1"/>
+      <c r="GX4" s="1"/>
+      <c r="GY4" s="1"/>
+      <c r="GZ4" s="1"/>
+      <c r="HA4" s="1"/>
+      <c r="HB4" s="1"/>
+      <c r="HC4" s="1"/>
+      <c r="HD4" s="1"/>
+      <c r="HE4" s="1"/>
+      <c r="HF4" s="1"/>
+      <c r="HG4" s="1"/>
+      <c r="HH4" s="1"/>
+      <c r="HI4" s="1"/>
+      <c r="HJ4" s="1"/>
+      <c r="HK4" s="1"/>
+      <c r="HL4" s="1"/>
+      <c r="HM4" s="1"/>
+      <c r="HN4" s="1"/>
+      <c r="HO4" s="1"/>
+      <c r="HP4" s="1"/>
+      <c r="HQ4" s="1"/>
+      <c r="HR4" s="1"/>
+      <c r="HS4" s="1"/>
+      <c r="HT4" s="1"/>
+      <c r="HU4" s="1"/>
+      <c r="HV4" s="1"/>
+      <c r="HW4" s="1"/>
+      <c r="HX4" s="1"/>
+      <c r="HY4" s="1"/>
+      <c r="HZ4" s="1"/>
+      <c r="IA4" s="1"/>
+      <c r="IB4" s="1"/>
+      <c r="IC4" s="1"/>
+      <c r="ID4" s="1"/>
+      <c r="IE4" s="1"/>
+      <c r="IF4" s="1"/>
+      <c r="IG4" s="1"/>
+      <c r="IH4" s="1"/>
+      <c r="II4" s="1"/>
+      <c r="IJ4" s="1"/>
+      <c r="IK4" s="1"/>
+      <c r="IL4" s="1"/>
+      <c r="IM4" s="1"/>
+      <c r="IN4" s="1"/>
+      <c r="IO4" s="1"/>
+      <c r="IP4" s="1"/>
+      <c r="IQ4" s="1"/>
+      <c r="IR4" s="1"/>
+      <c r="IS4" s="1"/>
+      <c r="IT4" s="1"/>
+      <c r="IU4" s="1"/>
+      <c r="IV4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
@@ -2989,7 +2995,7 @@
         <v>18</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -3308,78 +3314,78 @@
       <c r="FZ20" s="19"/>
       <c r="GA20" s="1"/>
       <c r="GB20" s="1"/>
-      <c r="GC20" s="0"/>
-      <c r="GD20" s="0"/>
-      <c r="GE20" s="0"/>
-      <c r="GF20" s="0"/>
-      <c r="GG20" s="0"/>
-      <c r="GH20" s="0"/>
-      <c r="GI20" s="0"/>
-      <c r="GJ20" s="0"/>
-      <c r="GK20" s="0"/>
-      <c r="GL20" s="0"/>
-      <c r="GM20" s="0"/>
-      <c r="GN20" s="0"/>
-      <c r="GO20" s="0"/>
-      <c r="GP20" s="0"/>
-      <c r="GQ20" s="0"/>
-      <c r="GR20" s="0"/>
-      <c r="GS20" s="0"/>
-      <c r="GT20" s="0"/>
-      <c r="GU20" s="0"/>
-      <c r="GV20" s="0"/>
-      <c r="GW20" s="0"/>
-      <c r="GX20" s="0"/>
-      <c r="GY20" s="0"/>
-      <c r="GZ20" s="0"/>
-      <c r="HA20" s="0"/>
-      <c r="HB20" s="0"/>
-      <c r="HC20" s="0"/>
-      <c r="HD20" s="0"/>
-      <c r="HE20" s="0"/>
-      <c r="HF20" s="0"/>
-      <c r="HG20" s="0"/>
-      <c r="HH20" s="0"/>
-      <c r="HI20" s="0"/>
-      <c r="HJ20" s="0"/>
-      <c r="HK20" s="0"/>
-      <c r="HL20" s="0"/>
-      <c r="HM20" s="0"/>
-      <c r="HN20" s="0"/>
-      <c r="HO20" s="0"/>
-      <c r="HP20" s="0"/>
-      <c r="HQ20" s="0"/>
-      <c r="HR20" s="0"/>
-      <c r="HS20" s="0"/>
-      <c r="HT20" s="0"/>
-      <c r="HU20" s="0"/>
-      <c r="HV20" s="0"/>
-      <c r="HW20" s="0"/>
-      <c r="HX20" s="0"/>
-      <c r="HY20" s="0"/>
-      <c r="HZ20" s="0"/>
-      <c r="IA20" s="0"/>
-      <c r="IB20" s="0"/>
-      <c r="IC20" s="0"/>
-      <c r="ID20" s="0"/>
-      <c r="IE20" s="0"/>
-      <c r="IF20" s="0"/>
-      <c r="IG20" s="0"/>
-      <c r="IH20" s="0"/>
-      <c r="II20" s="0"/>
-      <c r="IJ20" s="0"/>
-      <c r="IK20" s="0"/>
-      <c r="IL20" s="0"/>
-      <c r="IM20" s="0"/>
-      <c r="IN20" s="0"/>
-      <c r="IO20" s="0"/>
-      <c r="IP20" s="0"/>
-      <c r="IQ20" s="0"/>
-      <c r="IR20" s="0"/>
-      <c r="IS20" s="0"/>
-      <c r="IT20" s="0"/>
-      <c r="IU20" s="0"/>
-      <c r="IV20" s="0"/>
+      <c r="GC20" s="1"/>
+      <c r="GD20" s="1"/>
+      <c r="GE20" s="1"/>
+      <c r="GF20" s="1"/>
+      <c r="GG20" s="1"/>
+      <c r="GH20" s="1"/>
+      <c r="GI20" s="1"/>
+      <c r="GJ20" s="1"/>
+      <c r="GK20" s="1"/>
+      <c r="GL20" s="1"/>
+      <c r="GM20" s="1"/>
+      <c r="GN20" s="1"/>
+      <c r="GO20" s="1"/>
+      <c r="GP20" s="1"/>
+      <c r="GQ20" s="1"/>
+      <c r="GR20" s="1"/>
+      <c r="GS20" s="1"/>
+      <c r="GT20" s="1"/>
+      <c r="GU20" s="1"/>
+      <c r="GV20" s="1"/>
+      <c r="GW20" s="1"/>
+      <c r="GX20" s="1"/>
+      <c r="GY20" s="1"/>
+      <c r="GZ20" s="1"/>
+      <c r="HA20" s="1"/>
+      <c r="HB20" s="1"/>
+      <c r="HC20" s="1"/>
+      <c r="HD20" s="1"/>
+      <c r="HE20" s="1"/>
+      <c r="HF20" s="1"/>
+      <c r="HG20" s="1"/>
+      <c r="HH20" s="1"/>
+      <c r="HI20" s="1"/>
+      <c r="HJ20" s="1"/>
+      <c r="HK20" s="1"/>
+      <c r="HL20" s="1"/>
+      <c r="HM20" s="1"/>
+      <c r="HN20" s="1"/>
+      <c r="HO20" s="1"/>
+      <c r="HP20" s="1"/>
+      <c r="HQ20" s="1"/>
+      <c r="HR20" s="1"/>
+      <c r="HS20" s="1"/>
+      <c r="HT20" s="1"/>
+      <c r="HU20" s="1"/>
+      <c r="HV20" s="1"/>
+      <c r="HW20" s="1"/>
+      <c r="HX20" s="1"/>
+      <c r="HY20" s="1"/>
+      <c r="HZ20" s="1"/>
+      <c r="IA20" s="1"/>
+      <c r="IB20" s="1"/>
+      <c r="IC20" s="1"/>
+      <c r="ID20" s="1"/>
+      <c r="IE20" s="1"/>
+      <c r="IF20" s="1"/>
+      <c r="IG20" s="1"/>
+      <c r="IH20" s="1"/>
+      <c r="II20" s="1"/>
+      <c r="IJ20" s="1"/>
+      <c r="IK20" s="1"/>
+      <c r="IL20" s="1"/>
+      <c r="IM20" s="1"/>
+      <c r="IN20" s="1"/>
+      <c r="IO20" s="1"/>
+      <c r="IP20" s="1"/>
+      <c r="IQ20" s="1"/>
+      <c r="IR20" s="1"/>
+      <c r="IS20" s="1"/>
+      <c r="IT20" s="1"/>
+      <c r="IU20" s="1"/>
+      <c r="IV20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
@@ -3508,78 +3514,78 @@
       <c r="FZ24" s="1"/>
       <c r="GA24" s="1"/>
       <c r="GB24" s="1"/>
-      <c r="GC24" s="0"/>
-      <c r="GD24" s="0"/>
-      <c r="GE24" s="0"/>
-      <c r="GF24" s="0"/>
-      <c r="GG24" s="0"/>
-      <c r="GH24" s="0"/>
-      <c r="GI24" s="0"/>
-      <c r="GJ24" s="0"/>
-      <c r="GK24" s="0"/>
-      <c r="GL24" s="0"/>
-      <c r="GM24" s="0"/>
-      <c r="GN24" s="0"/>
-      <c r="GO24" s="0"/>
-      <c r="GP24" s="0"/>
-      <c r="GQ24" s="0"/>
-      <c r="GR24" s="0"/>
-      <c r="GS24" s="0"/>
-      <c r="GT24" s="0"/>
-      <c r="GU24" s="0"/>
-      <c r="GV24" s="0"/>
-      <c r="GW24" s="0"/>
-      <c r="GX24" s="0"/>
-      <c r="GY24" s="0"/>
-      <c r="GZ24" s="0"/>
-      <c r="HA24" s="0"/>
-      <c r="HB24" s="0"/>
-      <c r="HC24" s="0"/>
-      <c r="HD24" s="0"/>
-      <c r="HE24" s="0"/>
-      <c r="HF24" s="0"/>
-      <c r="HG24" s="0"/>
-      <c r="HH24" s="0"/>
-      <c r="HI24" s="0"/>
-      <c r="HJ24" s="0"/>
-      <c r="HK24" s="0"/>
-      <c r="HL24" s="0"/>
-      <c r="HM24" s="0"/>
-      <c r="HN24" s="0"/>
-      <c r="HO24" s="0"/>
-      <c r="HP24" s="0"/>
-      <c r="HQ24" s="0"/>
-      <c r="HR24" s="0"/>
-      <c r="HS24" s="0"/>
-      <c r="HT24" s="0"/>
-      <c r="HU24" s="0"/>
-      <c r="HV24" s="0"/>
-      <c r="HW24" s="0"/>
-      <c r="HX24" s="0"/>
-      <c r="HY24" s="0"/>
-      <c r="HZ24" s="0"/>
-      <c r="IA24" s="0"/>
-      <c r="IB24" s="0"/>
-      <c r="IC24" s="0"/>
-      <c r="ID24" s="0"/>
-      <c r="IE24" s="0"/>
-      <c r="IF24" s="0"/>
-      <c r="IG24" s="0"/>
-      <c r="IH24" s="0"/>
-      <c r="II24" s="0"/>
-      <c r="IJ24" s="0"/>
-      <c r="IK24" s="0"/>
-      <c r="IL24" s="0"/>
-      <c r="IM24" s="0"/>
-      <c r="IN24" s="0"/>
-      <c r="IO24" s="0"/>
-      <c r="IP24" s="0"/>
-      <c r="IQ24" s="0"/>
-      <c r="IR24" s="0"/>
-      <c r="IS24" s="0"/>
-      <c r="IT24" s="0"/>
-      <c r="IU24" s="0"/>
-      <c r="IV24" s="0"/>
+      <c r="GC24" s="1"/>
+      <c r="GD24" s="1"/>
+      <c r="GE24" s="1"/>
+      <c r="GF24" s="1"/>
+      <c r="GG24" s="1"/>
+      <c r="GH24" s="1"/>
+      <c r="GI24" s="1"/>
+      <c r="GJ24" s="1"/>
+      <c r="GK24" s="1"/>
+      <c r="GL24" s="1"/>
+      <c r="GM24" s="1"/>
+      <c r="GN24" s="1"/>
+      <c r="GO24" s="1"/>
+      <c r="GP24" s="1"/>
+      <c r="GQ24" s="1"/>
+      <c r="GR24" s="1"/>
+      <c r="GS24" s="1"/>
+      <c r="GT24" s="1"/>
+      <c r="GU24" s="1"/>
+      <c r="GV24" s="1"/>
+      <c r="GW24" s="1"/>
+      <c r="GX24" s="1"/>
+      <c r="GY24" s="1"/>
+      <c r="GZ24" s="1"/>
+      <c r="HA24" s="1"/>
+      <c r="HB24" s="1"/>
+      <c r="HC24" s="1"/>
+      <c r="HD24" s="1"/>
+      <c r="HE24" s="1"/>
+      <c r="HF24" s="1"/>
+      <c r="HG24" s="1"/>
+      <c r="HH24" s="1"/>
+      <c r="HI24" s="1"/>
+      <c r="HJ24" s="1"/>
+      <c r="HK24" s="1"/>
+      <c r="HL24" s="1"/>
+      <c r="HM24" s="1"/>
+      <c r="HN24" s="1"/>
+      <c r="HO24" s="1"/>
+      <c r="HP24" s="1"/>
+      <c r="HQ24" s="1"/>
+      <c r="HR24" s="1"/>
+      <c r="HS24" s="1"/>
+      <c r="HT24" s="1"/>
+      <c r="HU24" s="1"/>
+      <c r="HV24" s="1"/>
+      <c r="HW24" s="1"/>
+      <c r="HX24" s="1"/>
+      <c r="HY24" s="1"/>
+      <c r="HZ24" s="1"/>
+      <c r="IA24" s="1"/>
+      <c r="IB24" s="1"/>
+      <c r="IC24" s="1"/>
+      <c r="ID24" s="1"/>
+      <c r="IE24" s="1"/>
+      <c r="IF24" s="1"/>
+      <c r="IG24" s="1"/>
+      <c r="IH24" s="1"/>
+      <c r="II24" s="1"/>
+      <c r="IJ24" s="1"/>
+      <c r="IK24" s="1"/>
+      <c r="IL24" s="1"/>
+      <c r="IM24" s="1"/>
+      <c r="IN24" s="1"/>
+      <c r="IO24" s="1"/>
+      <c r="IP24" s="1"/>
+      <c r="IQ24" s="1"/>
+      <c r="IR24" s="1"/>
+      <c r="IS24" s="1"/>
+      <c r="IT24" s="1"/>
+      <c r="IU24" s="1"/>
+      <c r="IV24" s="1"/>
     </row>
     <row r="25" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
@@ -3828,78 +3834,78 @@
       <c r="FZ32" s="1"/>
       <c r="GA32" s="1"/>
       <c r="GB32" s="1"/>
-      <c r="GC32" s="0"/>
-      <c r="GD32" s="0"/>
-      <c r="GE32" s="0"/>
-      <c r="GF32" s="0"/>
-      <c r="GG32" s="0"/>
-      <c r="GH32" s="0"/>
-      <c r="GI32" s="0"/>
-      <c r="GJ32" s="0"/>
-      <c r="GK32" s="0"/>
-      <c r="GL32" s="0"/>
-      <c r="GM32" s="0"/>
-      <c r="GN32" s="0"/>
-      <c r="GO32" s="0"/>
-      <c r="GP32" s="0"/>
-      <c r="GQ32" s="0"/>
-      <c r="GR32" s="0"/>
-      <c r="GS32" s="0"/>
-      <c r="GT32" s="0"/>
-      <c r="GU32" s="0"/>
-      <c r="GV32" s="0"/>
-      <c r="GW32" s="0"/>
-      <c r="GX32" s="0"/>
-      <c r="GY32" s="0"/>
-      <c r="GZ32" s="0"/>
-      <c r="HA32" s="0"/>
-      <c r="HB32" s="0"/>
-      <c r="HC32" s="0"/>
-      <c r="HD32" s="0"/>
-      <c r="HE32" s="0"/>
-      <c r="HF32" s="0"/>
-      <c r="HG32" s="0"/>
-      <c r="HH32" s="0"/>
-      <c r="HI32" s="0"/>
-      <c r="HJ32" s="0"/>
-      <c r="HK32" s="0"/>
-      <c r="HL32" s="0"/>
-      <c r="HM32" s="0"/>
-      <c r="HN32" s="0"/>
-      <c r="HO32" s="0"/>
-      <c r="HP32" s="0"/>
-      <c r="HQ32" s="0"/>
-      <c r="HR32" s="0"/>
-      <c r="HS32" s="0"/>
-      <c r="HT32" s="0"/>
-      <c r="HU32" s="0"/>
-      <c r="HV32" s="0"/>
-      <c r="HW32" s="0"/>
-      <c r="HX32" s="0"/>
-      <c r="HY32" s="0"/>
-      <c r="HZ32" s="0"/>
-      <c r="IA32" s="0"/>
-      <c r="IB32" s="0"/>
-      <c r="IC32" s="0"/>
-      <c r="ID32" s="0"/>
-      <c r="IE32" s="0"/>
-      <c r="IF32" s="0"/>
-      <c r="IG32" s="0"/>
-      <c r="IH32" s="0"/>
-      <c r="II32" s="0"/>
-      <c r="IJ32" s="0"/>
-      <c r="IK32" s="0"/>
-      <c r="IL32" s="0"/>
-      <c r="IM32" s="0"/>
-      <c r="IN32" s="0"/>
-      <c r="IO32" s="0"/>
-      <c r="IP32" s="0"/>
-      <c r="IQ32" s="0"/>
-      <c r="IR32" s="0"/>
-      <c r="IS32" s="0"/>
-      <c r="IT32" s="0"/>
-      <c r="IU32" s="0"/>
-      <c r="IV32" s="0"/>
+      <c r="GC32" s="1"/>
+      <c r="GD32" s="1"/>
+      <c r="GE32" s="1"/>
+      <c r="GF32" s="1"/>
+      <c r="GG32" s="1"/>
+      <c r="GH32" s="1"/>
+      <c r="GI32" s="1"/>
+      <c r="GJ32" s="1"/>
+      <c r="GK32" s="1"/>
+      <c r="GL32" s="1"/>
+      <c r="GM32" s="1"/>
+      <c r="GN32" s="1"/>
+      <c r="GO32" s="1"/>
+      <c r="GP32" s="1"/>
+      <c r="GQ32" s="1"/>
+      <c r="GR32" s="1"/>
+      <c r="GS32" s="1"/>
+      <c r="GT32" s="1"/>
+      <c r="GU32" s="1"/>
+      <c r="GV32" s="1"/>
+      <c r="GW32" s="1"/>
+      <c r="GX32" s="1"/>
+      <c r="GY32" s="1"/>
+      <c r="GZ32" s="1"/>
+      <c r="HA32" s="1"/>
+      <c r="HB32" s="1"/>
+      <c r="HC32" s="1"/>
+      <c r="HD32" s="1"/>
+      <c r="HE32" s="1"/>
+      <c r="HF32" s="1"/>
+      <c r="HG32" s="1"/>
+      <c r="HH32" s="1"/>
+      <c r="HI32" s="1"/>
+      <c r="HJ32" s="1"/>
+      <c r="HK32" s="1"/>
+      <c r="HL32" s="1"/>
+      <c r="HM32" s="1"/>
+      <c r="HN32" s="1"/>
+      <c r="HO32" s="1"/>
+      <c r="HP32" s="1"/>
+      <c r="HQ32" s="1"/>
+      <c r="HR32" s="1"/>
+      <c r="HS32" s="1"/>
+      <c r="HT32" s="1"/>
+      <c r="HU32" s="1"/>
+      <c r="HV32" s="1"/>
+      <c r="HW32" s="1"/>
+      <c r="HX32" s="1"/>
+      <c r="HY32" s="1"/>
+      <c r="HZ32" s="1"/>
+      <c r="IA32" s="1"/>
+      <c r="IB32" s="1"/>
+      <c r="IC32" s="1"/>
+      <c r="ID32" s="1"/>
+      <c r="IE32" s="1"/>
+      <c r="IF32" s="1"/>
+      <c r="IG32" s="1"/>
+      <c r="IH32" s="1"/>
+      <c r="II32" s="1"/>
+      <c r="IJ32" s="1"/>
+      <c r="IK32" s="1"/>
+      <c r="IL32" s="1"/>
+      <c r="IM32" s="1"/>
+      <c r="IN32" s="1"/>
+      <c r="IO32" s="1"/>
+      <c r="IP32" s="1"/>
+      <c r="IQ32" s="1"/>
+      <c r="IR32" s="1"/>
+      <c r="IS32" s="1"/>
+      <c r="IT32" s="1"/>
+      <c r="IU32" s="1"/>
+      <c r="IV32" s="1"/>
     </row>
     <row r="33" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
@@ -4167,78 +4173,78 @@
       <c r="FZ35" s="1"/>
       <c r="GA35" s="1"/>
       <c r="GB35" s="1"/>
-      <c r="GC35" s="0"/>
-      <c r="GD35" s="0"/>
-      <c r="GE35" s="0"/>
-      <c r="GF35" s="0"/>
-      <c r="GG35" s="0"/>
-      <c r="GH35" s="0"/>
-      <c r="GI35" s="0"/>
-      <c r="GJ35" s="0"/>
-      <c r="GK35" s="0"/>
-      <c r="GL35" s="0"/>
-      <c r="GM35" s="0"/>
-      <c r="GN35" s="0"/>
-      <c r="GO35" s="0"/>
-      <c r="GP35" s="0"/>
-      <c r="GQ35" s="0"/>
-      <c r="GR35" s="0"/>
-      <c r="GS35" s="0"/>
-      <c r="GT35" s="0"/>
-      <c r="GU35" s="0"/>
-      <c r="GV35" s="0"/>
-      <c r="GW35" s="0"/>
-      <c r="GX35" s="0"/>
-      <c r="GY35" s="0"/>
-      <c r="GZ35" s="0"/>
-      <c r="HA35" s="0"/>
-      <c r="HB35" s="0"/>
-      <c r="HC35" s="0"/>
-      <c r="HD35" s="0"/>
-      <c r="HE35" s="0"/>
-      <c r="HF35" s="0"/>
-      <c r="HG35" s="0"/>
-      <c r="HH35" s="0"/>
-      <c r="HI35" s="0"/>
-      <c r="HJ35" s="0"/>
-      <c r="HK35" s="0"/>
-      <c r="HL35" s="0"/>
-      <c r="HM35" s="0"/>
-      <c r="HN35" s="0"/>
-      <c r="HO35" s="0"/>
-      <c r="HP35" s="0"/>
-      <c r="HQ35" s="0"/>
-      <c r="HR35" s="0"/>
-      <c r="HS35" s="0"/>
-      <c r="HT35" s="0"/>
-      <c r="HU35" s="0"/>
-      <c r="HV35" s="0"/>
-      <c r="HW35" s="0"/>
-      <c r="HX35" s="0"/>
-      <c r="HY35" s="0"/>
-      <c r="HZ35" s="0"/>
-      <c r="IA35" s="0"/>
-      <c r="IB35" s="0"/>
-      <c r="IC35" s="0"/>
-      <c r="ID35" s="0"/>
-      <c r="IE35" s="0"/>
-      <c r="IF35" s="0"/>
-      <c r="IG35" s="0"/>
-      <c r="IH35" s="0"/>
-      <c r="II35" s="0"/>
-      <c r="IJ35" s="0"/>
-      <c r="IK35" s="0"/>
-      <c r="IL35" s="0"/>
-      <c r="IM35" s="0"/>
-      <c r="IN35" s="0"/>
-      <c r="IO35" s="0"/>
-      <c r="IP35" s="0"/>
-      <c r="IQ35" s="0"/>
-      <c r="IR35" s="0"/>
-      <c r="IS35" s="0"/>
-      <c r="IT35" s="0"/>
-      <c r="IU35" s="0"/>
-      <c r="IV35" s="0"/>
+      <c r="GC35" s="1"/>
+      <c r="GD35" s="1"/>
+      <c r="GE35" s="1"/>
+      <c r="GF35" s="1"/>
+      <c r="GG35" s="1"/>
+      <c r="GH35" s="1"/>
+      <c r="GI35" s="1"/>
+      <c r="GJ35" s="1"/>
+      <c r="GK35" s="1"/>
+      <c r="GL35" s="1"/>
+      <c r="GM35" s="1"/>
+      <c r="GN35" s="1"/>
+      <c r="GO35" s="1"/>
+      <c r="GP35" s="1"/>
+      <c r="GQ35" s="1"/>
+      <c r="GR35" s="1"/>
+      <c r="GS35" s="1"/>
+      <c r="GT35" s="1"/>
+      <c r="GU35" s="1"/>
+      <c r="GV35" s="1"/>
+      <c r="GW35" s="1"/>
+      <c r="GX35" s="1"/>
+      <c r="GY35" s="1"/>
+      <c r="GZ35" s="1"/>
+      <c r="HA35" s="1"/>
+      <c r="HB35" s="1"/>
+      <c r="HC35" s="1"/>
+      <c r="HD35" s="1"/>
+      <c r="HE35" s="1"/>
+      <c r="HF35" s="1"/>
+      <c r="HG35" s="1"/>
+      <c r="HH35" s="1"/>
+      <c r="HI35" s="1"/>
+      <c r="HJ35" s="1"/>
+      <c r="HK35" s="1"/>
+      <c r="HL35" s="1"/>
+      <c r="HM35" s="1"/>
+      <c r="HN35" s="1"/>
+      <c r="HO35" s="1"/>
+      <c r="HP35" s="1"/>
+      <c r="HQ35" s="1"/>
+      <c r="HR35" s="1"/>
+      <c r="HS35" s="1"/>
+      <c r="HT35" s="1"/>
+      <c r="HU35" s="1"/>
+      <c r="HV35" s="1"/>
+      <c r="HW35" s="1"/>
+      <c r="HX35" s="1"/>
+      <c r="HY35" s="1"/>
+      <c r="HZ35" s="1"/>
+      <c r="IA35" s="1"/>
+      <c r="IB35" s="1"/>
+      <c r="IC35" s="1"/>
+      <c r="ID35" s="1"/>
+      <c r="IE35" s="1"/>
+      <c r="IF35" s="1"/>
+      <c r="IG35" s="1"/>
+      <c r="IH35" s="1"/>
+      <c r="II35" s="1"/>
+      <c r="IJ35" s="1"/>
+      <c r="IK35" s="1"/>
+      <c r="IL35" s="1"/>
+      <c r="IM35" s="1"/>
+      <c r="IN35" s="1"/>
+      <c r="IO35" s="1"/>
+      <c r="IP35" s="1"/>
+      <c r="IQ35" s="1"/>
+      <c r="IR35" s="1"/>
+      <c r="IS35" s="1"/>
+      <c r="IT35" s="1"/>
+      <c r="IU35" s="1"/>
+      <c r="IV35" s="1"/>
     </row>
     <row r="36" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
@@ -4412,78 +4418,78 @@
       <c r="FZ37" s="1"/>
       <c r="GA37" s="1"/>
       <c r="GB37" s="1"/>
-      <c r="GC37" s="0"/>
-      <c r="GD37" s="0"/>
-      <c r="GE37" s="0"/>
-      <c r="GF37" s="0"/>
-      <c r="GG37" s="0"/>
-      <c r="GH37" s="0"/>
-      <c r="GI37" s="0"/>
-      <c r="GJ37" s="0"/>
-      <c r="GK37" s="0"/>
-      <c r="GL37" s="0"/>
-      <c r="GM37" s="0"/>
-      <c r="GN37" s="0"/>
-      <c r="GO37" s="0"/>
-      <c r="GP37" s="0"/>
-      <c r="GQ37" s="0"/>
-      <c r="GR37" s="0"/>
-      <c r="GS37" s="0"/>
-      <c r="GT37" s="0"/>
-      <c r="GU37" s="0"/>
-      <c r="GV37" s="0"/>
-      <c r="GW37" s="0"/>
-      <c r="GX37" s="0"/>
-      <c r="GY37" s="0"/>
-      <c r="GZ37" s="0"/>
-      <c r="HA37" s="0"/>
-      <c r="HB37" s="0"/>
-      <c r="HC37" s="0"/>
-      <c r="HD37" s="0"/>
-      <c r="HE37" s="0"/>
-      <c r="HF37" s="0"/>
-      <c r="HG37" s="0"/>
-      <c r="HH37" s="0"/>
-      <c r="HI37" s="0"/>
-      <c r="HJ37" s="0"/>
-      <c r="HK37" s="0"/>
-      <c r="HL37" s="0"/>
-      <c r="HM37" s="0"/>
-      <c r="HN37" s="0"/>
-      <c r="HO37" s="0"/>
-      <c r="HP37" s="0"/>
-      <c r="HQ37" s="0"/>
-      <c r="HR37" s="0"/>
-      <c r="HS37" s="0"/>
-      <c r="HT37" s="0"/>
-      <c r="HU37" s="0"/>
-      <c r="HV37" s="0"/>
-      <c r="HW37" s="0"/>
-      <c r="HX37" s="0"/>
-      <c r="HY37" s="0"/>
-      <c r="HZ37" s="0"/>
-      <c r="IA37" s="0"/>
-      <c r="IB37" s="0"/>
-      <c r="IC37" s="0"/>
-      <c r="ID37" s="0"/>
-      <c r="IE37" s="0"/>
-      <c r="IF37" s="0"/>
-      <c r="IG37" s="0"/>
-      <c r="IH37" s="0"/>
-      <c r="II37" s="0"/>
-      <c r="IJ37" s="0"/>
-      <c r="IK37" s="0"/>
-      <c r="IL37" s="0"/>
-      <c r="IM37" s="0"/>
-      <c r="IN37" s="0"/>
-      <c r="IO37" s="0"/>
-      <c r="IP37" s="0"/>
-      <c r="IQ37" s="0"/>
-      <c r="IR37" s="0"/>
-      <c r="IS37" s="0"/>
-      <c r="IT37" s="0"/>
-      <c r="IU37" s="0"/>
-      <c r="IV37" s="0"/>
+      <c r="GC37" s="1"/>
+      <c r="GD37" s="1"/>
+      <c r="GE37" s="1"/>
+      <c r="GF37" s="1"/>
+      <c r="GG37" s="1"/>
+      <c r="GH37" s="1"/>
+      <c r="GI37" s="1"/>
+      <c r="GJ37" s="1"/>
+      <c r="GK37" s="1"/>
+      <c r="GL37" s="1"/>
+      <c r="GM37" s="1"/>
+      <c r="GN37" s="1"/>
+      <c r="GO37" s="1"/>
+      <c r="GP37" s="1"/>
+      <c r="GQ37" s="1"/>
+      <c r="GR37" s="1"/>
+      <c r="GS37" s="1"/>
+      <c r="GT37" s="1"/>
+      <c r="GU37" s="1"/>
+      <c r="GV37" s="1"/>
+      <c r="GW37" s="1"/>
+      <c r="GX37" s="1"/>
+      <c r="GY37" s="1"/>
+      <c r="GZ37" s="1"/>
+      <c r="HA37" s="1"/>
+      <c r="HB37" s="1"/>
+      <c r="HC37" s="1"/>
+      <c r="HD37" s="1"/>
+      <c r="HE37" s="1"/>
+      <c r="HF37" s="1"/>
+      <c r="HG37" s="1"/>
+      <c r="HH37" s="1"/>
+      <c r="HI37" s="1"/>
+      <c r="HJ37" s="1"/>
+      <c r="HK37" s="1"/>
+      <c r="HL37" s="1"/>
+      <c r="HM37" s="1"/>
+      <c r="HN37" s="1"/>
+      <c r="HO37" s="1"/>
+      <c r="HP37" s="1"/>
+      <c r="HQ37" s="1"/>
+      <c r="HR37" s="1"/>
+      <c r="HS37" s="1"/>
+      <c r="HT37" s="1"/>
+      <c r="HU37" s="1"/>
+      <c r="HV37" s="1"/>
+      <c r="HW37" s="1"/>
+      <c r="HX37" s="1"/>
+      <c r="HY37" s="1"/>
+      <c r="HZ37" s="1"/>
+      <c r="IA37" s="1"/>
+      <c r="IB37" s="1"/>
+      <c r="IC37" s="1"/>
+      <c r="ID37" s="1"/>
+      <c r="IE37" s="1"/>
+      <c r="IF37" s="1"/>
+      <c r="IG37" s="1"/>
+      <c r="IH37" s="1"/>
+      <c r="II37" s="1"/>
+      <c r="IJ37" s="1"/>
+      <c r="IK37" s="1"/>
+      <c r="IL37" s="1"/>
+      <c r="IM37" s="1"/>
+      <c r="IN37" s="1"/>
+      <c r="IO37" s="1"/>
+      <c r="IP37" s="1"/>
+      <c r="IQ37" s="1"/>
+      <c r="IR37" s="1"/>
+      <c r="IS37" s="1"/>
+      <c r="IT37" s="1"/>
+      <c r="IU37" s="1"/>
+      <c r="IV37" s="1"/>
     </row>
     <row r="38" s="19" customFormat="true" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
@@ -4597,78 +4603,78 @@
       <c r="FZ38" s="1"/>
       <c r="GA38" s="1"/>
       <c r="GB38" s="1"/>
-      <c r="GC38" s="0"/>
-      <c r="GD38" s="0"/>
-      <c r="GE38" s="0"/>
-      <c r="GF38" s="0"/>
-      <c r="GG38" s="0"/>
-      <c r="GH38" s="0"/>
-      <c r="GI38" s="0"/>
-      <c r="GJ38" s="0"/>
-      <c r="GK38" s="0"/>
-      <c r="GL38" s="0"/>
-      <c r="GM38" s="0"/>
-      <c r="GN38" s="0"/>
-      <c r="GO38" s="0"/>
-      <c r="GP38" s="0"/>
-      <c r="GQ38" s="0"/>
-      <c r="GR38" s="0"/>
-      <c r="GS38" s="0"/>
-      <c r="GT38" s="0"/>
-      <c r="GU38" s="0"/>
-      <c r="GV38" s="0"/>
-      <c r="GW38" s="0"/>
-      <c r="GX38" s="0"/>
-      <c r="GY38" s="0"/>
-      <c r="GZ38" s="0"/>
-      <c r="HA38" s="0"/>
-      <c r="HB38" s="0"/>
-      <c r="HC38" s="0"/>
-      <c r="HD38" s="0"/>
-      <c r="HE38" s="0"/>
-      <c r="HF38" s="0"/>
-      <c r="HG38" s="0"/>
-      <c r="HH38" s="0"/>
-      <c r="HI38" s="0"/>
-      <c r="HJ38" s="0"/>
-      <c r="HK38" s="0"/>
-      <c r="HL38" s="0"/>
-      <c r="HM38" s="0"/>
-      <c r="HN38" s="0"/>
-      <c r="HO38" s="0"/>
-      <c r="HP38" s="0"/>
-      <c r="HQ38" s="0"/>
-      <c r="HR38" s="0"/>
-      <c r="HS38" s="0"/>
-      <c r="HT38" s="0"/>
-      <c r="HU38" s="0"/>
-      <c r="HV38" s="0"/>
-      <c r="HW38" s="0"/>
-      <c r="HX38" s="0"/>
-      <c r="HY38" s="0"/>
-      <c r="HZ38" s="0"/>
-      <c r="IA38" s="0"/>
-      <c r="IB38" s="0"/>
-      <c r="IC38" s="0"/>
-      <c r="ID38" s="0"/>
-      <c r="IE38" s="0"/>
-      <c r="IF38" s="0"/>
-      <c r="IG38" s="0"/>
-      <c r="IH38" s="0"/>
-      <c r="II38" s="0"/>
-      <c r="IJ38" s="0"/>
-      <c r="IK38" s="0"/>
-      <c r="IL38" s="0"/>
-      <c r="IM38" s="0"/>
-      <c r="IN38" s="0"/>
-      <c r="IO38" s="0"/>
-      <c r="IP38" s="0"/>
-      <c r="IQ38" s="0"/>
-      <c r="IR38" s="0"/>
-      <c r="IS38" s="0"/>
-      <c r="IT38" s="0"/>
-      <c r="IU38" s="0"/>
-      <c r="IV38" s="0"/>
+      <c r="GC38" s="1"/>
+      <c r="GD38" s="1"/>
+      <c r="GE38" s="1"/>
+      <c r="GF38" s="1"/>
+      <c r="GG38" s="1"/>
+      <c r="GH38" s="1"/>
+      <c r="GI38" s="1"/>
+      <c r="GJ38" s="1"/>
+      <c r="GK38" s="1"/>
+      <c r="GL38" s="1"/>
+      <c r="GM38" s="1"/>
+      <c r="GN38" s="1"/>
+      <c r="GO38" s="1"/>
+      <c r="GP38" s="1"/>
+      <c r="GQ38" s="1"/>
+      <c r="GR38" s="1"/>
+      <c r="GS38" s="1"/>
+      <c r="GT38" s="1"/>
+      <c r="GU38" s="1"/>
+      <c r="GV38" s="1"/>
+      <c r="GW38" s="1"/>
+      <c r="GX38" s="1"/>
+      <c r="GY38" s="1"/>
+      <c r="GZ38" s="1"/>
+      <c r="HA38" s="1"/>
+      <c r="HB38" s="1"/>
+      <c r="HC38" s="1"/>
+      <c r="HD38" s="1"/>
+      <c r="HE38" s="1"/>
+      <c r="HF38" s="1"/>
+      <c r="HG38" s="1"/>
+      <c r="HH38" s="1"/>
+      <c r="HI38" s="1"/>
+      <c r="HJ38" s="1"/>
+      <c r="HK38" s="1"/>
+      <c r="HL38" s="1"/>
+      <c r="HM38" s="1"/>
+      <c r="HN38" s="1"/>
+      <c r="HO38" s="1"/>
+      <c r="HP38" s="1"/>
+      <c r="HQ38" s="1"/>
+      <c r="HR38" s="1"/>
+      <c r="HS38" s="1"/>
+      <c r="HT38" s="1"/>
+      <c r="HU38" s="1"/>
+      <c r="HV38" s="1"/>
+      <c r="HW38" s="1"/>
+      <c r="HX38" s="1"/>
+      <c r="HY38" s="1"/>
+      <c r="HZ38" s="1"/>
+      <c r="IA38" s="1"/>
+      <c r="IB38" s="1"/>
+      <c r="IC38" s="1"/>
+      <c r="ID38" s="1"/>
+      <c r="IE38" s="1"/>
+      <c r="IF38" s="1"/>
+      <c r="IG38" s="1"/>
+      <c r="IH38" s="1"/>
+      <c r="II38" s="1"/>
+      <c r="IJ38" s="1"/>
+      <c r="IK38" s="1"/>
+      <c r="IL38" s="1"/>
+      <c r="IM38" s="1"/>
+      <c r="IN38" s="1"/>
+      <c r="IO38" s="1"/>
+      <c r="IP38" s="1"/>
+      <c r="IQ38" s="1"/>
+      <c r="IR38" s="1"/>
+      <c r="IS38" s="1"/>
+      <c r="IT38" s="1"/>
+      <c r="IU38" s="1"/>
+      <c r="IV38" s="1"/>
     </row>
     <row r="39" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="15" t="s">
@@ -5024,78 +5030,78 @@
       <c r="FZ42" s="1"/>
       <c r="GA42" s="1"/>
       <c r="GB42" s="1"/>
-      <c r="GC42" s="0"/>
-      <c r="GD42" s="0"/>
-      <c r="GE42" s="0"/>
-      <c r="GF42" s="0"/>
-      <c r="GG42" s="0"/>
-      <c r="GH42" s="0"/>
-      <c r="GI42" s="0"/>
-      <c r="GJ42" s="0"/>
-      <c r="GK42" s="0"/>
-      <c r="GL42" s="0"/>
-      <c r="GM42" s="0"/>
-      <c r="GN42" s="0"/>
-      <c r="GO42" s="0"/>
-      <c r="GP42" s="0"/>
-      <c r="GQ42" s="0"/>
-      <c r="GR42" s="0"/>
-      <c r="GS42" s="0"/>
-      <c r="GT42" s="0"/>
-      <c r="GU42" s="0"/>
-      <c r="GV42" s="0"/>
-      <c r="GW42" s="0"/>
-      <c r="GX42" s="0"/>
-      <c r="GY42" s="0"/>
-      <c r="GZ42" s="0"/>
-      <c r="HA42" s="0"/>
-      <c r="HB42" s="0"/>
-      <c r="HC42" s="0"/>
-      <c r="HD42" s="0"/>
-      <c r="HE42" s="0"/>
-      <c r="HF42" s="0"/>
-      <c r="HG42" s="0"/>
-      <c r="HH42" s="0"/>
-      <c r="HI42" s="0"/>
-      <c r="HJ42" s="0"/>
-      <c r="HK42" s="0"/>
-      <c r="HL42" s="0"/>
-      <c r="HM42" s="0"/>
-      <c r="HN42" s="0"/>
-      <c r="HO42" s="0"/>
-      <c r="HP42" s="0"/>
-      <c r="HQ42" s="0"/>
-      <c r="HR42" s="0"/>
-      <c r="HS42" s="0"/>
-      <c r="HT42" s="0"/>
-      <c r="HU42" s="0"/>
-      <c r="HV42" s="0"/>
-      <c r="HW42" s="0"/>
-      <c r="HX42" s="0"/>
-      <c r="HY42" s="0"/>
-      <c r="HZ42" s="0"/>
-      <c r="IA42" s="0"/>
-      <c r="IB42" s="0"/>
-      <c r="IC42" s="0"/>
-      <c r="ID42" s="0"/>
-      <c r="IE42" s="0"/>
-      <c r="IF42" s="0"/>
-      <c r="IG42" s="0"/>
-      <c r="IH42" s="0"/>
-      <c r="II42" s="0"/>
-      <c r="IJ42" s="0"/>
-      <c r="IK42" s="0"/>
-      <c r="IL42" s="0"/>
-      <c r="IM42" s="0"/>
-      <c r="IN42" s="0"/>
-      <c r="IO42" s="0"/>
-      <c r="IP42" s="0"/>
-      <c r="IQ42" s="0"/>
-      <c r="IR42" s="0"/>
-      <c r="IS42" s="0"/>
-      <c r="IT42" s="0"/>
-      <c r="IU42" s="0"/>
-      <c r="IV42" s="0"/>
+      <c r="GC42" s="1"/>
+      <c r="GD42" s="1"/>
+      <c r="GE42" s="1"/>
+      <c r="GF42" s="1"/>
+      <c r="GG42" s="1"/>
+      <c r="GH42" s="1"/>
+      <c r="GI42" s="1"/>
+      <c r="GJ42" s="1"/>
+      <c r="GK42" s="1"/>
+      <c r="GL42" s="1"/>
+      <c r="GM42" s="1"/>
+      <c r="GN42" s="1"/>
+      <c r="GO42" s="1"/>
+      <c r="GP42" s="1"/>
+      <c r="GQ42" s="1"/>
+      <c r="GR42" s="1"/>
+      <c r="GS42" s="1"/>
+      <c r="GT42" s="1"/>
+      <c r="GU42" s="1"/>
+      <c r="GV42" s="1"/>
+      <c r="GW42" s="1"/>
+      <c r="GX42" s="1"/>
+      <c r="GY42" s="1"/>
+      <c r="GZ42" s="1"/>
+      <c r="HA42" s="1"/>
+      <c r="HB42" s="1"/>
+      <c r="HC42" s="1"/>
+      <c r="HD42" s="1"/>
+      <c r="HE42" s="1"/>
+      <c r="HF42" s="1"/>
+      <c r="HG42" s="1"/>
+      <c r="HH42" s="1"/>
+      <c r="HI42" s="1"/>
+      <c r="HJ42" s="1"/>
+      <c r="HK42" s="1"/>
+      <c r="HL42" s="1"/>
+      <c r="HM42" s="1"/>
+      <c r="HN42" s="1"/>
+      <c r="HO42" s="1"/>
+      <c r="HP42" s="1"/>
+      <c r="HQ42" s="1"/>
+      <c r="HR42" s="1"/>
+      <c r="HS42" s="1"/>
+      <c r="HT42" s="1"/>
+      <c r="HU42" s="1"/>
+      <c r="HV42" s="1"/>
+      <c r="HW42" s="1"/>
+      <c r="HX42" s="1"/>
+      <c r="HY42" s="1"/>
+      <c r="HZ42" s="1"/>
+      <c r="IA42" s="1"/>
+      <c r="IB42" s="1"/>
+      <c r="IC42" s="1"/>
+      <c r="ID42" s="1"/>
+      <c r="IE42" s="1"/>
+      <c r="IF42" s="1"/>
+      <c r="IG42" s="1"/>
+      <c r="IH42" s="1"/>
+      <c r="II42" s="1"/>
+      <c r="IJ42" s="1"/>
+      <c r="IK42" s="1"/>
+      <c r="IL42" s="1"/>
+      <c r="IM42" s="1"/>
+      <c r="IN42" s="1"/>
+      <c r="IO42" s="1"/>
+      <c r="IP42" s="1"/>
+      <c r="IQ42" s="1"/>
+      <c r="IR42" s="1"/>
+      <c r="IS42" s="1"/>
+      <c r="IT42" s="1"/>
+      <c r="IU42" s="1"/>
+      <c r="IV42" s="1"/>
     </row>
     <row r="43" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="15"/>
@@ -6297,78 +6303,78 @@
       <c r="FZ58" s="1"/>
       <c r="GA58" s="1"/>
       <c r="GB58" s="1"/>
-      <c r="GC58" s="0"/>
-      <c r="GD58" s="0"/>
-      <c r="GE58" s="0"/>
-      <c r="GF58" s="0"/>
-      <c r="GG58" s="0"/>
-      <c r="GH58" s="0"/>
-      <c r="GI58" s="0"/>
-      <c r="GJ58" s="0"/>
-      <c r="GK58" s="0"/>
-      <c r="GL58" s="0"/>
-      <c r="GM58" s="0"/>
-      <c r="GN58" s="0"/>
-      <c r="GO58" s="0"/>
-      <c r="GP58" s="0"/>
-      <c r="GQ58" s="0"/>
-      <c r="GR58" s="0"/>
-      <c r="GS58" s="0"/>
-      <c r="GT58" s="0"/>
-      <c r="GU58" s="0"/>
-      <c r="GV58" s="0"/>
-      <c r="GW58" s="0"/>
-      <c r="GX58" s="0"/>
-      <c r="GY58" s="0"/>
-      <c r="GZ58" s="0"/>
-      <c r="HA58" s="0"/>
-      <c r="HB58" s="0"/>
-      <c r="HC58" s="0"/>
-      <c r="HD58" s="0"/>
-      <c r="HE58" s="0"/>
-      <c r="HF58" s="0"/>
-      <c r="HG58" s="0"/>
-      <c r="HH58" s="0"/>
-      <c r="HI58" s="0"/>
-      <c r="HJ58" s="0"/>
-      <c r="HK58" s="0"/>
-      <c r="HL58" s="0"/>
-      <c r="HM58" s="0"/>
-      <c r="HN58" s="0"/>
-      <c r="HO58" s="0"/>
-      <c r="HP58" s="0"/>
-      <c r="HQ58" s="0"/>
-      <c r="HR58" s="0"/>
-      <c r="HS58" s="0"/>
-      <c r="HT58" s="0"/>
-      <c r="HU58" s="0"/>
-      <c r="HV58" s="0"/>
-      <c r="HW58" s="0"/>
-      <c r="HX58" s="0"/>
-      <c r="HY58" s="0"/>
-      <c r="HZ58" s="0"/>
-      <c r="IA58" s="0"/>
-      <c r="IB58" s="0"/>
-      <c r="IC58" s="0"/>
-      <c r="ID58" s="0"/>
-      <c r="IE58" s="0"/>
-      <c r="IF58" s="0"/>
-      <c r="IG58" s="0"/>
-      <c r="IH58" s="0"/>
-      <c r="II58" s="0"/>
-      <c r="IJ58" s="0"/>
-      <c r="IK58" s="0"/>
-      <c r="IL58" s="0"/>
-      <c r="IM58" s="0"/>
-      <c r="IN58" s="0"/>
-      <c r="IO58" s="0"/>
-      <c r="IP58" s="0"/>
-      <c r="IQ58" s="0"/>
-      <c r="IR58" s="0"/>
-      <c r="IS58" s="0"/>
-      <c r="IT58" s="0"/>
-      <c r="IU58" s="0"/>
-      <c r="IV58" s="0"/>
+      <c r="GC58" s="1"/>
+      <c r="GD58" s="1"/>
+      <c r="GE58" s="1"/>
+      <c r="GF58" s="1"/>
+      <c r="GG58" s="1"/>
+      <c r="GH58" s="1"/>
+      <c r="GI58" s="1"/>
+      <c r="GJ58" s="1"/>
+      <c r="GK58" s="1"/>
+      <c r="GL58" s="1"/>
+      <c r="GM58" s="1"/>
+      <c r="GN58" s="1"/>
+      <c r="GO58" s="1"/>
+      <c r="GP58" s="1"/>
+      <c r="GQ58" s="1"/>
+      <c r="GR58" s="1"/>
+      <c r="GS58" s="1"/>
+      <c r="GT58" s="1"/>
+      <c r="GU58" s="1"/>
+      <c r="GV58" s="1"/>
+      <c r="GW58" s="1"/>
+      <c r="GX58" s="1"/>
+      <c r="GY58" s="1"/>
+      <c r="GZ58" s="1"/>
+      <c r="HA58" s="1"/>
+      <c r="HB58" s="1"/>
+      <c r="HC58" s="1"/>
+      <c r="HD58" s="1"/>
+      <c r="HE58" s="1"/>
+      <c r="HF58" s="1"/>
+      <c r="HG58" s="1"/>
+      <c r="HH58" s="1"/>
+      <c r="HI58" s="1"/>
+      <c r="HJ58" s="1"/>
+      <c r="HK58" s="1"/>
+      <c r="HL58" s="1"/>
+      <c r="HM58" s="1"/>
+      <c r="HN58" s="1"/>
+      <c r="HO58" s="1"/>
+      <c r="HP58" s="1"/>
+      <c r="HQ58" s="1"/>
+      <c r="HR58" s="1"/>
+      <c r="HS58" s="1"/>
+      <c r="HT58" s="1"/>
+      <c r="HU58" s="1"/>
+      <c r="HV58" s="1"/>
+      <c r="HW58" s="1"/>
+      <c r="HX58" s="1"/>
+      <c r="HY58" s="1"/>
+      <c r="HZ58" s="1"/>
+      <c r="IA58" s="1"/>
+      <c r="IB58" s="1"/>
+      <c r="IC58" s="1"/>
+      <c r="ID58" s="1"/>
+      <c r="IE58" s="1"/>
+      <c r="IF58" s="1"/>
+      <c r="IG58" s="1"/>
+      <c r="IH58" s="1"/>
+      <c r="II58" s="1"/>
+      <c r="IJ58" s="1"/>
+      <c r="IK58" s="1"/>
+      <c r="IL58" s="1"/>
+      <c r="IM58" s="1"/>
+      <c r="IN58" s="1"/>
+      <c r="IO58" s="1"/>
+      <c r="IP58" s="1"/>
+      <c r="IQ58" s="1"/>
+      <c r="IR58" s="1"/>
+      <c r="IS58" s="1"/>
+      <c r="IT58" s="1"/>
+      <c r="IU58" s="1"/>
+      <c r="IV58" s="1"/>
     </row>
     <row r="59" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="15"/>
@@ -6629,78 +6635,78 @@
       <c r="FZ61" s="1"/>
       <c r="GA61" s="1"/>
       <c r="GB61" s="1"/>
-      <c r="GC61" s="0"/>
-      <c r="GD61" s="0"/>
-      <c r="GE61" s="0"/>
-      <c r="GF61" s="0"/>
-      <c r="GG61" s="0"/>
-      <c r="GH61" s="0"/>
-      <c r="GI61" s="0"/>
-      <c r="GJ61" s="0"/>
-      <c r="GK61" s="0"/>
-      <c r="GL61" s="0"/>
-      <c r="GM61" s="0"/>
-      <c r="GN61" s="0"/>
-      <c r="GO61" s="0"/>
-      <c r="GP61" s="0"/>
-      <c r="GQ61" s="0"/>
-      <c r="GR61" s="0"/>
-      <c r="GS61" s="0"/>
-      <c r="GT61" s="0"/>
-      <c r="GU61" s="0"/>
-      <c r="GV61" s="0"/>
-      <c r="GW61" s="0"/>
-      <c r="GX61" s="0"/>
-      <c r="GY61" s="0"/>
-      <c r="GZ61" s="0"/>
-      <c r="HA61" s="0"/>
-      <c r="HB61" s="0"/>
-      <c r="HC61" s="0"/>
-      <c r="HD61" s="0"/>
-      <c r="HE61" s="0"/>
-      <c r="HF61" s="0"/>
-      <c r="HG61" s="0"/>
-      <c r="HH61" s="0"/>
-      <c r="HI61" s="0"/>
-      <c r="HJ61" s="0"/>
-      <c r="HK61" s="0"/>
-      <c r="HL61" s="0"/>
-      <c r="HM61" s="0"/>
-      <c r="HN61" s="0"/>
-      <c r="HO61" s="0"/>
-      <c r="HP61" s="0"/>
-      <c r="HQ61" s="0"/>
-      <c r="HR61" s="0"/>
-      <c r="HS61" s="0"/>
-      <c r="HT61" s="0"/>
-      <c r="HU61" s="0"/>
-      <c r="HV61" s="0"/>
-      <c r="HW61" s="0"/>
-      <c r="HX61" s="0"/>
-      <c r="HY61" s="0"/>
-      <c r="HZ61" s="0"/>
-      <c r="IA61" s="0"/>
-      <c r="IB61" s="0"/>
-      <c r="IC61" s="0"/>
-      <c r="ID61" s="0"/>
-      <c r="IE61" s="0"/>
-      <c r="IF61" s="0"/>
-      <c r="IG61" s="0"/>
-      <c r="IH61" s="0"/>
-      <c r="II61" s="0"/>
-      <c r="IJ61" s="0"/>
-      <c r="IK61" s="0"/>
-      <c r="IL61" s="0"/>
-      <c r="IM61" s="0"/>
-      <c r="IN61" s="0"/>
-      <c r="IO61" s="0"/>
-      <c r="IP61" s="0"/>
-      <c r="IQ61" s="0"/>
-      <c r="IR61" s="0"/>
-      <c r="IS61" s="0"/>
-      <c r="IT61" s="0"/>
-      <c r="IU61" s="0"/>
-      <c r="IV61" s="0"/>
+      <c r="GC61" s="1"/>
+      <c r="GD61" s="1"/>
+      <c r="GE61" s="1"/>
+      <c r="GF61" s="1"/>
+      <c r="GG61" s="1"/>
+      <c r="GH61" s="1"/>
+      <c r="GI61" s="1"/>
+      <c r="GJ61" s="1"/>
+      <c r="GK61" s="1"/>
+      <c r="GL61" s="1"/>
+      <c r="GM61" s="1"/>
+      <c r="GN61" s="1"/>
+      <c r="GO61" s="1"/>
+      <c r="GP61" s="1"/>
+      <c r="GQ61" s="1"/>
+      <c r="GR61" s="1"/>
+      <c r="GS61" s="1"/>
+      <c r="GT61" s="1"/>
+      <c r="GU61" s="1"/>
+      <c r="GV61" s="1"/>
+      <c r="GW61" s="1"/>
+      <c r="GX61" s="1"/>
+      <c r="GY61" s="1"/>
+      <c r="GZ61" s="1"/>
+      <c r="HA61" s="1"/>
+      <c r="HB61" s="1"/>
+      <c r="HC61" s="1"/>
+      <c r="HD61" s="1"/>
+      <c r="HE61" s="1"/>
+      <c r="HF61" s="1"/>
+      <c r="HG61" s="1"/>
+      <c r="HH61" s="1"/>
+      <c r="HI61" s="1"/>
+      <c r="HJ61" s="1"/>
+      <c r="HK61" s="1"/>
+      <c r="HL61" s="1"/>
+      <c r="HM61" s="1"/>
+      <c r="HN61" s="1"/>
+      <c r="HO61" s="1"/>
+      <c r="HP61" s="1"/>
+      <c r="HQ61" s="1"/>
+      <c r="HR61" s="1"/>
+      <c r="HS61" s="1"/>
+      <c r="HT61" s="1"/>
+      <c r="HU61" s="1"/>
+      <c r="HV61" s="1"/>
+      <c r="HW61" s="1"/>
+      <c r="HX61" s="1"/>
+      <c r="HY61" s="1"/>
+      <c r="HZ61" s="1"/>
+      <c r="IA61" s="1"/>
+      <c r="IB61" s="1"/>
+      <c r="IC61" s="1"/>
+      <c r="ID61" s="1"/>
+      <c r="IE61" s="1"/>
+      <c r="IF61" s="1"/>
+      <c r="IG61" s="1"/>
+      <c r="IH61" s="1"/>
+      <c r="II61" s="1"/>
+      <c r="IJ61" s="1"/>
+      <c r="IK61" s="1"/>
+      <c r="IL61" s="1"/>
+      <c r="IM61" s="1"/>
+      <c r="IN61" s="1"/>
+      <c r="IO61" s="1"/>
+      <c r="IP61" s="1"/>
+      <c r="IQ61" s="1"/>
+      <c r="IR61" s="1"/>
+      <c r="IS61" s="1"/>
+      <c r="IT61" s="1"/>
+      <c r="IU61" s="1"/>
+      <c r="IV61" s="1"/>
     </row>
     <row r="62" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11"/>
@@ -6863,78 +6869,78 @@
       <c r="FP63" s="1"/>
       <c r="GA63" s="1"/>
       <c r="GB63" s="1"/>
-      <c r="GC63" s="0"/>
-      <c r="GD63" s="0"/>
-      <c r="GE63" s="0"/>
-      <c r="GF63" s="0"/>
-      <c r="GG63" s="0"/>
-      <c r="GH63" s="0"/>
-      <c r="GI63" s="0"/>
-      <c r="GJ63" s="0"/>
-      <c r="GK63" s="0"/>
-      <c r="GL63" s="0"/>
-      <c r="GM63" s="0"/>
-      <c r="GN63" s="0"/>
-      <c r="GO63" s="0"/>
-      <c r="GP63" s="0"/>
-      <c r="GQ63" s="0"/>
-      <c r="GR63" s="0"/>
-      <c r="GS63" s="0"/>
-      <c r="GT63" s="0"/>
-      <c r="GU63" s="0"/>
-      <c r="GV63" s="0"/>
-      <c r="GW63" s="0"/>
-      <c r="GX63" s="0"/>
-      <c r="GY63" s="0"/>
-      <c r="GZ63" s="0"/>
-      <c r="HA63" s="0"/>
-      <c r="HB63" s="0"/>
-      <c r="HC63" s="0"/>
-      <c r="HD63" s="0"/>
-      <c r="HE63" s="0"/>
-      <c r="HF63" s="0"/>
-      <c r="HG63" s="0"/>
-      <c r="HH63" s="0"/>
-      <c r="HI63" s="0"/>
-      <c r="HJ63" s="0"/>
-      <c r="HK63" s="0"/>
-      <c r="HL63" s="0"/>
-      <c r="HM63" s="0"/>
-      <c r="HN63" s="0"/>
-      <c r="HO63" s="0"/>
-      <c r="HP63" s="0"/>
-      <c r="HQ63" s="0"/>
-      <c r="HR63" s="0"/>
-      <c r="HS63" s="0"/>
-      <c r="HT63" s="0"/>
-      <c r="HU63" s="0"/>
-      <c r="HV63" s="0"/>
-      <c r="HW63" s="0"/>
-      <c r="HX63" s="0"/>
-      <c r="HY63" s="0"/>
-      <c r="HZ63" s="0"/>
-      <c r="IA63" s="0"/>
-      <c r="IB63" s="0"/>
-      <c r="IC63" s="0"/>
-      <c r="ID63" s="0"/>
-      <c r="IE63" s="0"/>
-      <c r="IF63" s="0"/>
-      <c r="IG63" s="0"/>
-      <c r="IH63" s="0"/>
-      <c r="II63" s="0"/>
-      <c r="IJ63" s="0"/>
-      <c r="IK63" s="0"/>
-      <c r="IL63" s="0"/>
-      <c r="IM63" s="0"/>
-      <c r="IN63" s="0"/>
-      <c r="IO63" s="0"/>
-      <c r="IP63" s="0"/>
-      <c r="IQ63" s="0"/>
-      <c r="IR63" s="0"/>
-      <c r="IS63" s="0"/>
-      <c r="IT63" s="0"/>
-      <c r="IU63" s="0"/>
-      <c r="IV63" s="0"/>
+      <c r="GC63" s="1"/>
+      <c r="GD63" s="1"/>
+      <c r="GE63" s="1"/>
+      <c r="GF63" s="1"/>
+      <c r="GG63" s="1"/>
+      <c r="GH63" s="1"/>
+      <c r="GI63" s="1"/>
+      <c r="GJ63" s="1"/>
+      <c r="GK63" s="1"/>
+      <c r="GL63" s="1"/>
+      <c r="GM63" s="1"/>
+      <c r="GN63" s="1"/>
+      <c r="GO63" s="1"/>
+      <c r="GP63" s="1"/>
+      <c r="GQ63" s="1"/>
+      <c r="GR63" s="1"/>
+      <c r="GS63" s="1"/>
+      <c r="GT63" s="1"/>
+      <c r="GU63" s="1"/>
+      <c r="GV63" s="1"/>
+      <c r="GW63" s="1"/>
+      <c r="GX63" s="1"/>
+      <c r="GY63" s="1"/>
+      <c r="GZ63" s="1"/>
+      <c r="HA63" s="1"/>
+      <c r="HB63" s="1"/>
+      <c r="HC63" s="1"/>
+      <c r="HD63" s="1"/>
+      <c r="HE63" s="1"/>
+      <c r="HF63" s="1"/>
+      <c r="HG63" s="1"/>
+      <c r="HH63" s="1"/>
+      <c r="HI63" s="1"/>
+      <c r="HJ63" s="1"/>
+      <c r="HK63" s="1"/>
+      <c r="HL63" s="1"/>
+      <c r="HM63" s="1"/>
+      <c r="HN63" s="1"/>
+      <c r="HO63" s="1"/>
+      <c r="HP63" s="1"/>
+      <c r="HQ63" s="1"/>
+      <c r="HR63" s="1"/>
+      <c r="HS63" s="1"/>
+      <c r="HT63" s="1"/>
+      <c r="HU63" s="1"/>
+      <c r="HV63" s="1"/>
+      <c r="HW63" s="1"/>
+      <c r="HX63" s="1"/>
+      <c r="HY63" s="1"/>
+      <c r="HZ63" s="1"/>
+      <c r="IA63" s="1"/>
+      <c r="IB63" s="1"/>
+      <c r="IC63" s="1"/>
+      <c r="ID63" s="1"/>
+      <c r="IE63" s="1"/>
+      <c r="IF63" s="1"/>
+      <c r="IG63" s="1"/>
+      <c r="IH63" s="1"/>
+      <c r="II63" s="1"/>
+      <c r="IJ63" s="1"/>
+      <c r="IK63" s="1"/>
+      <c r="IL63" s="1"/>
+      <c r="IM63" s="1"/>
+      <c r="IN63" s="1"/>
+      <c r="IO63" s="1"/>
+      <c r="IP63" s="1"/>
+      <c r="IQ63" s="1"/>
+      <c r="IR63" s="1"/>
+      <c r="IS63" s="1"/>
+      <c r="IT63" s="1"/>
+      <c r="IU63" s="1"/>
+      <c r="IV63" s="1"/>
     </row>
     <row r="64" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="11"/>
@@ -7316,78 +7322,78 @@
       <c r="FZ68" s="1"/>
       <c r="GA68" s="1"/>
       <c r="GB68" s="1"/>
-      <c r="GC68" s="0"/>
-      <c r="GD68" s="0"/>
-      <c r="GE68" s="0"/>
-      <c r="GF68" s="0"/>
-      <c r="GG68" s="0"/>
-      <c r="GH68" s="0"/>
-      <c r="GI68" s="0"/>
-      <c r="GJ68" s="0"/>
-      <c r="GK68" s="0"/>
-      <c r="GL68" s="0"/>
-      <c r="GM68" s="0"/>
-      <c r="GN68" s="0"/>
-      <c r="GO68" s="0"/>
-      <c r="GP68" s="0"/>
-      <c r="GQ68" s="0"/>
-      <c r="GR68" s="0"/>
-      <c r="GS68" s="0"/>
-      <c r="GT68" s="0"/>
-      <c r="GU68" s="0"/>
-      <c r="GV68" s="0"/>
-      <c r="GW68" s="0"/>
-      <c r="GX68" s="0"/>
-      <c r="GY68" s="0"/>
-      <c r="GZ68" s="0"/>
-      <c r="HA68" s="0"/>
-      <c r="HB68" s="0"/>
-      <c r="HC68" s="0"/>
-      <c r="HD68" s="0"/>
-      <c r="HE68" s="0"/>
-      <c r="HF68" s="0"/>
-      <c r="HG68" s="0"/>
-      <c r="HH68" s="0"/>
-      <c r="HI68" s="0"/>
-      <c r="HJ68" s="0"/>
-      <c r="HK68" s="0"/>
-      <c r="HL68" s="0"/>
-      <c r="HM68" s="0"/>
-      <c r="HN68" s="0"/>
-      <c r="HO68" s="0"/>
-      <c r="HP68" s="0"/>
-      <c r="HQ68" s="0"/>
-      <c r="HR68" s="0"/>
-      <c r="HS68" s="0"/>
-      <c r="HT68" s="0"/>
-      <c r="HU68" s="0"/>
-      <c r="HV68" s="0"/>
-      <c r="HW68" s="0"/>
-      <c r="HX68" s="0"/>
-      <c r="HY68" s="0"/>
-      <c r="HZ68" s="0"/>
-      <c r="IA68" s="0"/>
-      <c r="IB68" s="0"/>
-      <c r="IC68" s="0"/>
-      <c r="ID68" s="0"/>
-      <c r="IE68" s="0"/>
-      <c r="IF68" s="0"/>
-      <c r="IG68" s="0"/>
-      <c r="IH68" s="0"/>
-      <c r="II68" s="0"/>
-      <c r="IJ68" s="0"/>
-      <c r="IK68" s="0"/>
-      <c r="IL68" s="0"/>
-      <c r="IM68" s="0"/>
-      <c r="IN68" s="0"/>
-      <c r="IO68" s="0"/>
-      <c r="IP68" s="0"/>
-      <c r="IQ68" s="0"/>
-      <c r="IR68" s="0"/>
-      <c r="IS68" s="0"/>
-      <c r="IT68" s="0"/>
-      <c r="IU68" s="0"/>
-      <c r="IV68" s="0"/>
+      <c r="GC68" s="1"/>
+      <c r="GD68" s="1"/>
+      <c r="GE68" s="1"/>
+      <c r="GF68" s="1"/>
+      <c r="GG68" s="1"/>
+      <c r="GH68" s="1"/>
+      <c r="GI68" s="1"/>
+      <c r="GJ68" s="1"/>
+      <c r="GK68" s="1"/>
+      <c r="GL68" s="1"/>
+      <c r="GM68" s="1"/>
+      <c r="GN68" s="1"/>
+      <c r="GO68" s="1"/>
+      <c r="GP68" s="1"/>
+      <c r="GQ68" s="1"/>
+      <c r="GR68" s="1"/>
+      <c r="GS68" s="1"/>
+      <c r="GT68" s="1"/>
+      <c r="GU68" s="1"/>
+      <c r="GV68" s="1"/>
+      <c r="GW68" s="1"/>
+      <c r="GX68" s="1"/>
+      <c r="GY68" s="1"/>
+      <c r="GZ68" s="1"/>
+      <c r="HA68" s="1"/>
+      <c r="HB68" s="1"/>
+      <c r="HC68" s="1"/>
+      <c r="HD68" s="1"/>
+      <c r="HE68" s="1"/>
+      <c r="HF68" s="1"/>
+      <c r="HG68" s="1"/>
+      <c r="HH68" s="1"/>
+      <c r="HI68" s="1"/>
+      <c r="HJ68" s="1"/>
+      <c r="HK68" s="1"/>
+      <c r="HL68" s="1"/>
+      <c r="HM68" s="1"/>
+      <c r="HN68" s="1"/>
+      <c r="HO68" s="1"/>
+      <c r="HP68" s="1"/>
+      <c r="HQ68" s="1"/>
+      <c r="HR68" s="1"/>
+      <c r="HS68" s="1"/>
+      <c r="HT68" s="1"/>
+      <c r="HU68" s="1"/>
+      <c r="HV68" s="1"/>
+      <c r="HW68" s="1"/>
+      <c r="HX68" s="1"/>
+      <c r="HY68" s="1"/>
+      <c r="HZ68" s="1"/>
+      <c r="IA68" s="1"/>
+      <c r="IB68" s="1"/>
+      <c r="IC68" s="1"/>
+      <c r="ID68" s="1"/>
+      <c r="IE68" s="1"/>
+      <c r="IF68" s="1"/>
+      <c r="IG68" s="1"/>
+      <c r="IH68" s="1"/>
+      <c r="II68" s="1"/>
+      <c r="IJ68" s="1"/>
+      <c r="IK68" s="1"/>
+      <c r="IL68" s="1"/>
+      <c r="IM68" s="1"/>
+      <c r="IN68" s="1"/>
+      <c r="IO68" s="1"/>
+      <c r="IP68" s="1"/>
+      <c r="IQ68" s="1"/>
+      <c r="IR68" s="1"/>
+      <c r="IS68" s="1"/>
+      <c r="IT68" s="1"/>
+      <c r="IU68" s="1"/>
+      <c r="IV68" s="1"/>
     </row>
     <row r="69" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="15"/>
@@ -8315,78 +8321,78 @@
       <c r="FZ80" s="1"/>
       <c r="GA80" s="1"/>
       <c r="GB80" s="1"/>
-      <c r="GC80" s="0"/>
-      <c r="GD80" s="0"/>
-      <c r="GE80" s="0"/>
-      <c r="GF80" s="0"/>
-      <c r="GG80" s="0"/>
-      <c r="GH80" s="0"/>
-      <c r="GI80" s="0"/>
-      <c r="GJ80" s="0"/>
-      <c r="GK80" s="0"/>
-      <c r="GL80" s="0"/>
-      <c r="GM80" s="0"/>
-      <c r="GN80" s="0"/>
-      <c r="GO80" s="0"/>
-      <c r="GP80" s="0"/>
-      <c r="GQ80" s="0"/>
-      <c r="GR80" s="0"/>
-      <c r="GS80" s="0"/>
-      <c r="GT80" s="0"/>
-      <c r="GU80" s="0"/>
-      <c r="GV80" s="0"/>
-      <c r="GW80" s="0"/>
-      <c r="GX80" s="0"/>
-      <c r="GY80" s="0"/>
-      <c r="GZ80" s="0"/>
-      <c r="HA80" s="0"/>
-      <c r="HB80" s="0"/>
-      <c r="HC80" s="0"/>
-      <c r="HD80" s="0"/>
-      <c r="HE80" s="0"/>
-      <c r="HF80" s="0"/>
-      <c r="HG80" s="0"/>
-      <c r="HH80" s="0"/>
-      <c r="HI80" s="0"/>
-      <c r="HJ80" s="0"/>
-      <c r="HK80" s="0"/>
-      <c r="HL80" s="0"/>
-      <c r="HM80" s="0"/>
-      <c r="HN80" s="0"/>
-      <c r="HO80" s="0"/>
-      <c r="HP80" s="0"/>
-      <c r="HQ80" s="0"/>
-      <c r="HR80" s="0"/>
-      <c r="HS80" s="0"/>
-      <c r="HT80" s="0"/>
-      <c r="HU80" s="0"/>
-      <c r="HV80" s="0"/>
-      <c r="HW80" s="0"/>
-      <c r="HX80" s="0"/>
-      <c r="HY80" s="0"/>
-      <c r="HZ80" s="0"/>
-      <c r="IA80" s="0"/>
-      <c r="IB80" s="0"/>
-      <c r="IC80" s="0"/>
-      <c r="ID80" s="0"/>
-      <c r="IE80" s="0"/>
-      <c r="IF80" s="0"/>
-      <c r="IG80" s="0"/>
-      <c r="IH80" s="0"/>
-      <c r="II80" s="0"/>
-      <c r="IJ80" s="0"/>
-      <c r="IK80" s="0"/>
-      <c r="IL80" s="0"/>
-      <c r="IM80" s="0"/>
-      <c r="IN80" s="0"/>
-      <c r="IO80" s="0"/>
-      <c r="IP80" s="0"/>
-      <c r="IQ80" s="0"/>
-      <c r="IR80" s="0"/>
-      <c r="IS80" s="0"/>
-      <c r="IT80" s="0"/>
-      <c r="IU80" s="0"/>
-      <c r="IV80" s="0"/>
+      <c r="GC80" s="1"/>
+      <c r="GD80" s="1"/>
+      <c r="GE80" s="1"/>
+      <c r="GF80" s="1"/>
+      <c r="GG80" s="1"/>
+      <c r="GH80" s="1"/>
+      <c r="GI80" s="1"/>
+      <c r="GJ80" s="1"/>
+      <c r="GK80" s="1"/>
+      <c r="GL80" s="1"/>
+      <c r="GM80" s="1"/>
+      <c r="GN80" s="1"/>
+      <c r="GO80" s="1"/>
+      <c r="GP80" s="1"/>
+      <c r="GQ80" s="1"/>
+      <c r="GR80" s="1"/>
+      <c r="GS80" s="1"/>
+      <c r="GT80" s="1"/>
+      <c r="GU80" s="1"/>
+      <c r="GV80" s="1"/>
+      <c r="GW80" s="1"/>
+      <c r="GX80" s="1"/>
+      <c r="GY80" s="1"/>
+      <c r="GZ80" s="1"/>
+      <c r="HA80" s="1"/>
+      <c r="HB80" s="1"/>
+      <c r="HC80" s="1"/>
+      <c r="HD80" s="1"/>
+      <c r="HE80" s="1"/>
+      <c r="HF80" s="1"/>
+      <c r="HG80" s="1"/>
+      <c r="HH80" s="1"/>
+      <c r="HI80" s="1"/>
+      <c r="HJ80" s="1"/>
+      <c r="HK80" s="1"/>
+      <c r="HL80" s="1"/>
+      <c r="HM80" s="1"/>
+      <c r="HN80" s="1"/>
+      <c r="HO80" s="1"/>
+      <c r="HP80" s="1"/>
+      <c r="HQ80" s="1"/>
+      <c r="HR80" s="1"/>
+      <c r="HS80" s="1"/>
+      <c r="HT80" s="1"/>
+      <c r="HU80" s="1"/>
+      <c r="HV80" s="1"/>
+      <c r="HW80" s="1"/>
+      <c r="HX80" s="1"/>
+      <c r="HY80" s="1"/>
+      <c r="HZ80" s="1"/>
+      <c r="IA80" s="1"/>
+      <c r="IB80" s="1"/>
+      <c r="IC80" s="1"/>
+      <c r="ID80" s="1"/>
+      <c r="IE80" s="1"/>
+      <c r="IF80" s="1"/>
+      <c r="IG80" s="1"/>
+      <c r="IH80" s="1"/>
+      <c r="II80" s="1"/>
+      <c r="IJ80" s="1"/>
+      <c r="IK80" s="1"/>
+      <c r="IL80" s="1"/>
+      <c r="IM80" s="1"/>
+      <c r="IN80" s="1"/>
+      <c r="IO80" s="1"/>
+      <c r="IP80" s="1"/>
+      <c r="IQ80" s="1"/>
+      <c r="IR80" s="1"/>
+      <c r="IS80" s="1"/>
+      <c r="IT80" s="1"/>
+      <c r="IU80" s="1"/>
+      <c r="IV80" s="1"/>
     </row>
     <row r="81" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="15"/>
@@ -9216,78 +9222,78 @@
       <c r="FZ91" s="1"/>
       <c r="GA91" s="1"/>
       <c r="GB91" s="1"/>
-      <c r="GC91" s="0"/>
-      <c r="GD91" s="0"/>
-      <c r="GE91" s="0"/>
-      <c r="GF91" s="0"/>
-      <c r="GG91" s="0"/>
-      <c r="GH91" s="0"/>
-      <c r="GI91" s="0"/>
-      <c r="GJ91" s="0"/>
-      <c r="GK91" s="0"/>
-      <c r="GL91" s="0"/>
-      <c r="GM91" s="0"/>
-      <c r="GN91" s="0"/>
-      <c r="GO91" s="0"/>
-      <c r="GP91" s="0"/>
-      <c r="GQ91" s="0"/>
-      <c r="GR91" s="0"/>
-      <c r="GS91" s="0"/>
-      <c r="GT91" s="0"/>
-      <c r="GU91" s="0"/>
-      <c r="GV91" s="0"/>
-      <c r="GW91" s="0"/>
-      <c r="GX91" s="0"/>
-      <c r="GY91" s="0"/>
-      <c r="GZ91" s="0"/>
-      <c r="HA91" s="0"/>
-      <c r="HB91" s="0"/>
-      <c r="HC91" s="0"/>
-      <c r="HD91" s="0"/>
-      <c r="HE91" s="0"/>
-      <c r="HF91" s="0"/>
-      <c r="HG91" s="0"/>
-      <c r="HH91" s="0"/>
-      <c r="HI91" s="0"/>
-      <c r="HJ91" s="0"/>
-      <c r="HK91" s="0"/>
-      <c r="HL91" s="0"/>
-      <c r="HM91" s="0"/>
-      <c r="HN91" s="0"/>
-      <c r="HO91" s="0"/>
-      <c r="HP91" s="0"/>
-      <c r="HQ91" s="0"/>
-      <c r="HR91" s="0"/>
-      <c r="HS91" s="0"/>
-      <c r="HT91" s="0"/>
-      <c r="HU91" s="0"/>
-      <c r="HV91" s="0"/>
-      <c r="HW91" s="0"/>
-      <c r="HX91" s="0"/>
-      <c r="HY91" s="0"/>
-      <c r="HZ91" s="0"/>
-      <c r="IA91" s="0"/>
-      <c r="IB91" s="0"/>
-      <c r="IC91" s="0"/>
-      <c r="ID91" s="0"/>
-      <c r="IE91" s="0"/>
-      <c r="IF91" s="0"/>
-      <c r="IG91" s="0"/>
-      <c r="IH91" s="0"/>
-      <c r="II91" s="0"/>
-      <c r="IJ91" s="0"/>
-      <c r="IK91" s="0"/>
-      <c r="IL91" s="0"/>
-      <c r="IM91" s="0"/>
-      <c r="IN91" s="0"/>
-      <c r="IO91" s="0"/>
-      <c r="IP91" s="0"/>
-      <c r="IQ91" s="0"/>
-      <c r="IR91" s="0"/>
-      <c r="IS91" s="0"/>
-      <c r="IT91" s="0"/>
-      <c r="IU91" s="0"/>
-      <c r="IV91" s="0"/>
+      <c r="GC91" s="1"/>
+      <c r="GD91" s="1"/>
+      <c r="GE91" s="1"/>
+      <c r="GF91" s="1"/>
+      <c r="GG91" s="1"/>
+      <c r="GH91" s="1"/>
+      <c r="GI91" s="1"/>
+      <c r="GJ91" s="1"/>
+      <c r="GK91" s="1"/>
+      <c r="GL91" s="1"/>
+      <c r="GM91" s="1"/>
+      <c r="GN91" s="1"/>
+      <c r="GO91" s="1"/>
+      <c r="GP91" s="1"/>
+      <c r="GQ91" s="1"/>
+      <c r="GR91" s="1"/>
+      <c r="GS91" s="1"/>
+      <c r="GT91" s="1"/>
+      <c r="GU91" s="1"/>
+      <c r="GV91" s="1"/>
+      <c r="GW91" s="1"/>
+      <c r="GX91" s="1"/>
+      <c r="GY91" s="1"/>
+      <c r="GZ91" s="1"/>
+      <c r="HA91" s="1"/>
+      <c r="HB91" s="1"/>
+      <c r="HC91" s="1"/>
+      <c r="HD91" s="1"/>
+      <c r="HE91" s="1"/>
+      <c r="HF91" s="1"/>
+      <c r="HG91" s="1"/>
+      <c r="HH91" s="1"/>
+      <c r="HI91" s="1"/>
+      <c r="HJ91" s="1"/>
+      <c r="HK91" s="1"/>
+      <c r="HL91" s="1"/>
+      <c r="HM91" s="1"/>
+      <c r="HN91" s="1"/>
+      <c r="HO91" s="1"/>
+      <c r="HP91" s="1"/>
+      <c r="HQ91" s="1"/>
+      <c r="HR91" s="1"/>
+      <c r="HS91" s="1"/>
+      <c r="HT91" s="1"/>
+      <c r="HU91" s="1"/>
+      <c r="HV91" s="1"/>
+      <c r="HW91" s="1"/>
+      <c r="HX91" s="1"/>
+      <c r="HY91" s="1"/>
+      <c r="HZ91" s="1"/>
+      <c r="IA91" s="1"/>
+      <c r="IB91" s="1"/>
+      <c r="IC91" s="1"/>
+      <c r="ID91" s="1"/>
+      <c r="IE91" s="1"/>
+      <c r="IF91" s="1"/>
+      <c r="IG91" s="1"/>
+      <c r="IH91" s="1"/>
+      <c r="II91" s="1"/>
+      <c r="IJ91" s="1"/>
+      <c r="IK91" s="1"/>
+      <c r="IL91" s="1"/>
+      <c r="IM91" s="1"/>
+      <c r="IN91" s="1"/>
+      <c r="IO91" s="1"/>
+      <c r="IP91" s="1"/>
+      <c r="IQ91" s="1"/>
+      <c r="IR91" s="1"/>
+      <c r="IS91" s="1"/>
+      <c r="IT91" s="1"/>
+      <c r="IU91" s="1"/>
+      <c r="IV91" s="1"/>
     </row>
     <row r="92" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="11"/>
@@ -9739,78 +9745,78 @@
       <c r="FZ97" s="1"/>
       <c r="GA97" s="1"/>
       <c r="GB97" s="1"/>
-      <c r="GC97" s="0"/>
-      <c r="GD97" s="0"/>
-      <c r="GE97" s="0"/>
-      <c r="GF97" s="0"/>
-      <c r="GG97" s="0"/>
-      <c r="GH97" s="0"/>
-      <c r="GI97" s="0"/>
-      <c r="GJ97" s="0"/>
-      <c r="GK97" s="0"/>
-      <c r="GL97" s="0"/>
-      <c r="GM97" s="0"/>
-      <c r="GN97" s="0"/>
-      <c r="GO97" s="0"/>
-      <c r="GP97" s="0"/>
-      <c r="GQ97" s="0"/>
-      <c r="GR97" s="0"/>
-      <c r="GS97" s="0"/>
-      <c r="GT97" s="0"/>
-      <c r="GU97" s="0"/>
-      <c r="GV97" s="0"/>
-      <c r="GW97" s="0"/>
-      <c r="GX97" s="0"/>
-      <c r="GY97" s="0"/>
-      <c r="GZ97" s="0"/>
-      <c r="HA97" s="0"/>
-      <c r="HB97" s="0"/>
-      <c r="HC97" s="0"/>
-      <c r="HD97" s="0"/>
-      <c r="HE97" s="0"/>
-      <c r="HF97" s="0"/>
-      <c r="HG97" s="0"/>
-      <c r="HH97" s="0"/>
-      <c r="HI97" s="0"/>
-      <c r="HJ97" s="0"/>
-      <c r="HK97" s="0"/>
-      <c r="HL97" s="0"/>
-      <c r="HM97" s="0"/>
-      <c r="HN97" s="0"/>
-      <c r="HO97" s="0"/>
-      <c r="HP97" s="0"/>
-      <c r="HQ97" s="0"/>
-      <c r="HR97" s="0"/>
-      <c r="HS97" s="0"/>
-      <c r="HT97" s="0"/>
-      <c r="HU97" s="0"/>
-      <c r="HV97" s="0"/>
-      <c r="HW97" s="0"/>
-      <c r="HX97" s="0"/>
-      <c r="HY97" s="0"/>
-      <c r="HZ97" s="0"/>
-      <c r="IA97" s="0"/>
-      <c r="IB97" s="0"/>
-      <c r="IC97" s="0"/>
-      <c r="ID97" s="0"/>
-      <c r="IE97" s="0"/>
-      <c r="IF97" s="0"/>
-      <c r="IG97" s="0"/>
-      <c r="IH97" s="0"/>
-      <c r="II97" s="0"/>
-      <c r="IJ97" s="0"/>
-      <c r="IK97" s="0"/>
-      <c r="IL97" s="0"/>
-      <c r="IM97" s="0"/>
-      <c r="IN97" s="0"/>
-      <c r="IO97" s="0"/>
-      <c r="IP97" s="0"/>
-      <c r="IQ97" s="0"/>
-      <c r="IR97" s="0"/>
-      <c r="IS97" s="0"/>
-      <c r="IT97" s="0"/>
-      <c r="IU97" s="0"/>
-      <c r="IV97" s="0"/>
+      <c r="GC97" s="1"/>
+      <c r="GD97" s="1"/>
+      <c r="GE97" s="1"/>
+      <c r="GF97" s="1"/>
+      <c r="GG97" s="1"/>
+      <c r="GH97" s="1"/>
+      <c r="GI97" s="1"/>
+      <c r="GJ97" s="1"/>
+      <c r="GK97" s="1"/>
+      <c r="GL97" s="1"/>
+      <c r="GM97" s="1"/>
+      <c r="GN97" s="1"/>
+      <c r="GO97" s="1"/>
+      <c r="GP97" s="1"/>
+      <c r="GQ97" s="1"/>
+      <c r="GR97" s="1"/>
+      <c r="GS97" s="1"/>
+      <c r="GT97" s="1"/>
+      <c r="GU97" s="1"/>
+      <c r="GV97" s="1"/>
+      <c r="GW97" s="1"/>
+      <c r="GX97" s="1"/>
+      <c r="GY97" s="1"/>
+      <c r="GZ97" s="1"/>
+      <c r="HA97" s="1"/>
+      <c r="HB97" s="1"/>
+      <c r="HC97" s="1"/>
+      <c r="HD97" s="1"/>
+      <c r="HE97" s="1"/>
+      <c r="HF97" s="1"/>
+      <c r="HG97" s="1"/>
+      <c r="HH97" s="1"/>
+      <c r="HI97" s="1"/>
+      <c r="HJ97" s="1"/>
+      <c r="HK97" s="1"/>
+      <c r="HL97" s="1"/>
+      <c r="HM97" s="1"/>
+      <c r="HN97" s="1"/>
+      <c r="HO97" s="1"/>
+      <c r="HP97" s="1"/>
+      <c r="HQ97" s="1"/>
+      <c r="HR97" s="1"/>
+      <c r="HS97" s="1"/>
+      <c r="HT97" s="1"/>
+      <c r="HU97" s="1"/>
+      <c r="HV97" s="1"/>
+      <c r="HW97" s="1"/>
+      <c r="HX97" s="1"/>
+      <c r="HY97" s="1"/>
+      <c r="HZ97" s="1"/>
+      <c r="IA97" s="1"/>
+      <c r="IB97" s="1"/>
+      <c r="IC97" s="1"/>
+      <c r="ID97" s="1"/>
+      <c r="IE97" s="1"/>
+      <c r="IF97" s="1"/>
+      <c r="IG97" s="1"/>
+      <c r="IH97" s="1"/>
+      <c r="II97" s="1"/>
+      <c r="IJ97" s="1"/>
+      <c r="IK97" s="1"/>
+      <c r="IL97" s="1"/>
+      <c r="IM97" s="1"/>
+      <c r="IN97" s="1"/>
+      <c r="IO97" s="1"/>
+      <c r="IP97" s="1"/>
+      <c r="IQ97" s="1"/>
+      <c r="IR97" s="1"/>
+      <c r="IS97" s="1"/>
+      <c r="IT97" s="1"/>
+      <c r="IU97" s="1"/>
+      <c r="IV97" s="1"/>
     </row>
     <row r="98" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="11"/>
@@ -10332,78 +10338,78 @@
       <c r="FZ104" s="1"/>
       <c r="GA104" s="1"/>
       <c r="GB104" s="1"/>
-      <c r="GC104" s="0"/>
-      <c r="GD104" s="0"/>
-      <c r="GE104" s="0"/>
-      <c r="GF104" s="0"/>
-      <c r="GG104" s="0"/>
-      <c r="GH104" s="0"/>
-      <c r="GI104" s="0"/>
-      <c r="GJ104" s="0"/>
-      <c r="GK104" s="0"/>
-      <c r="GL104" s="0"/>
-      <c r="GM104" s="0"/>
-      <c r="GN104" s="0"/>
-      <c r="GO104" s="0"/>
-      <c r="GP104" s="0"/>
-      <c r="GQ104" s="0"/>
-      <c r="GR104" s="0"/>
-      <c r="GS104" s="0"/>
-      <c r="GT104" s="0"/>
-      <c r="GU104" s="0"/>
-      <c r="GV104" s="0"/>
-      <c r="GW104" s="0"/>
-      <c r="GX104" s="0"/>
-      <c r="GY104" s="0"/>
-      <c r="GZ104" s="0"/>
-      <c r="HA104" s="0"/>
-      <c r="HB104" s="0"/>
-      <c r="HC104" s="0"/>
-      <c r="HD104" s="0"/>
-      <c r="HE104" s="0"/>
-      <c r="HF104" s="0"/>
-      <c r="HG104" s="0"/>
-      <c r="HH104" s="0"/>
-      <c r="HI104" s="0"/>
-      <c r="HJ104" s="0"/>
-      <c r="HK104" s="0"/>
-      <c r="HL104" s="0"/>
-      <c r="HM104" s="0"/>
-      <c r="HN104" s="0"/>
-      <c r="HO104" s="0"/>
-      <c r="HP104" s="0"/>
-      <c r="HQ104" s="0"/>
-      <c r="HR104" s="0"/>
-      <c r="HS104" s="0"/>
-      <c r="HT104" s="0"/>
-      <c r="HU104" s="0"/>
-      <c r="HV104" s="0"/>
-      <c r="HW104" s="0"/>
-      <c r="HX104" s="0"/>
-      <c r="HY104" s="0"/>
-      <c r="HZ104" s="0"/>
-      <c r="IA104" s="0"/>
-      <c r="IB104" s="0"/>
-      <c r="IC104" s="0"/>
-      <c r="ID104" s="0"/>
-      <c r="IE104" s="0"/>
-      <c r="IF104" s="0"/>
-      <c r="IG104" s="0"/>
-      <c r="IH104" s="0"/>
-      <c r="II104" s="0"/>
-      <c r="IJ104" s="0"/>
-      <c r="IK104" s="0"/>
-      <c r="IL104" s="0"/>
-      <c r="IM104" s="0"/>
-      <c r="IN104" s="0"/>
-      <c r="IO104" s="0"/>
-      <c r="IP104" s="0"/>
-      <c r="IQ104" s="0"/>
-      <c r="IR104" s="0"/>
-      <c r="IS104" s="0"/>
-      <c r="IT104" s="0"/>
-      <c r="IU104" s="0"/>
-      <c r="IV104" s="0"/>
+      <c r="GC104" s="1"/>
+      <c r="GD104" s="1"/>
+      <c r="GE104" s="1"/>
+      <c r="GF104" s="1"/>
+      <c r="GG104" s="1"/>
+      <c r="GH104" s="1"/>
+      <c r="GI104" s="1"/>
+      <c r="GJ104" s="1"/>
+      <c r="GK104" s="1"/>
+      <c r="GL104" s="1"/>
+      <c r="GM104" s="1"/>
+      <c r="GN104" s="1"/>
+      <c r="GO104" s="1"/>
+      <c r="GP104" s="1"/>
+      <c r="GQ104" s="1"/>
+      <c r="GR104" s="1"/>
+      <c r="GS104" s="1"/>
+      <c r="GT104" s="1"/>
+      <c r="GU104" s="1"/>
+      <c r="GV104" s="1"/>
+      <c r="GW104" s="1"/>
+      <c r="GX104" s="1"/>
+      <c r="GY104" s="1"/>
+      <c r="GZ104" s="1"/>
+      <c r="HA104" s="1"/>
+      <c r="HB104" s="1"/>
+      <c r="HC104" s="1"/>
+      <c r="HD104" s="1"/>
+      <c r="HE104" s="1"/>
+      <c r="HF104" s="1"/>
+      <c r="HG104" s="1"/>
+      <c r="HH104" s="1"/>
+      <c r="HI104" s="1"/>
+      <c r="HJ104" s="1"/>
+      <c r="HK104" s="1"/>
+      <c r="HL104" s="1"/>
+      <c r="HM104" s="1"/>
+      <c r="HN104" s="1"/>
+      <c r="HO104" s="1"/>
+      <c r="HP104" s="1"/>
+      <c r="HQ104" s="1"/>
+      <c r="HR104" s="1"/>
+      <c r="HS104" s="1"/>
+      <c r="HT104" s="1"/>
+      <c r="HU104" s="1"/>
+      <c r="HV104" s="1"/>
+      <c r="HW104" s="1"/>
+      <c r="HX104" s="1"/>
+      <c r="HY104" s="1"/>
+      <c r="HZ104" s="1"/>
+      <c r="IA104" s="1"/>
+      <c r="IB104" s="1"/>
+      <c r="IC104" s="1"/>
+      <c r="ID104" s="1"/>
+      <c r="IE104" s="1"/>
+      <c r="IF104" s="1"/>
+      <c r="IG104" s="1"/>
+      <c r="IH104" s="1"/>
+      <c r="II104" s="1"/>
+      <c r="IJ104" s="1"/>
+      <c r="IK104" s="1"/>
+      <c r="IL104" s="1"/>
+      <c r="IM104" s="1"/>
+      <c r="IN104" s="1"/>
+      <c r="IO104" s="1"/>
+      <c r="IP104" s="1"/>
+      <c r="IQ104" s="1"/>
+      <c r="IR104" s="1"/>
+      <c r="IS104" s="1"/>
+      <c r="IT104" s="1"/>
+      <c r="IU104" s="1"/>
+      <c r="IV104" s="1"/>
     </row>
     <row r="105" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="15"/>

</xml_diff>